<commit_message>
docs(schedule): 補上組員B T-030~T-037 狀態格底色與字色
文字已在上一筆改為 ✅ 已完成，本筆補齊 4 個分頁共 28 格
的底色（淡綠 #CE9ACD→RGB 13561798）與字色（深綠 24832），
與其他已完成任務格式一致。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Lucky_Star_Casino\Lucky_Star_Casino\Lucky_Star_Casino\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94B91D76-24A6-4185-A271-401EE312793A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{307F58F2-3628-4AFE-849D-6C9A6F7E5572}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1338,7 +1338,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1434,8 +1434,14 @@
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="19">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1524,6 +1530,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -1631,7 +1643,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1760,20 +1772,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1791,6 +1803,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -3009,7 +3027,7 @@
       <c r="I31" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="J31" s="31" t="s">
+      <c r="J31" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -3041,7 +3059,7 @@
       <c r="I32" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="J32" s="31" t="s">
+      <c r="J32" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -3073,7 +3091,7 @@
       <c r="I33" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J33" s="31" t="s">
+      <c r="J33" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -3105,7 +3123,7 @@
       <c r="I34" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="J34" s="31" t="s">
+      <c r="J34" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -5495,7 +5513,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="54" t="s">
         <v>354</v>
       </c>
       <c r="B1" s="53"/>
@@ -6087,7 +6105,7 @@
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A22" s="54" t="s">
+      <c r="A22" s="52" t="s">
         <v>355</v>
       </c>
       <c r="B22" s="53"/>
@@ -6102,7 +6120,7 @@
       </c>
     </row>
     <row r="24" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="54" t="s">
         <v>356</v>
       </c>
       <c r="B24" s="53"/>
@@ -6167,8 +6185,8 @@
       <c r="H26" s="13">
         <v>6</v>
       </c>
-      <c r="I26" s="31" t="s">
-        <v>431</v>
+      <c r="I26" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -6196,8 +6214,8 @@
       <c r="H27" s="13">
         <v>8</v>
       </c>
-      <c r="I27" s="31" t="s">
-        <v>431</v>
+      <c r="I27" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -6225,8 +6243,8 @@
       <c r="H28" s="13">
         <v>6</v>
       </c>
-      <c r="I28" s="31" t="s">
-        <v>431</v>
+      <c r="I28" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -6254,8 +6272,8 @@
       <c r="H29" s="13">
         <v>3</v>
       </c>
-      <c r="I29" s="31" t="s">
-        <v>431</v>
+      <c r="I29" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -6283,8 +6301,8 @@
       <c r="H30" s="15">
         <v>8</v>
       </c>
-      <c r="I30" s="31" t="s">
-        <v>431</v>
+      <c r="I30" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -6312,8 +6330,8 @@
       <c r="H31" s="15">
         <v>5</v>
       </c>
-      <c r="I31" s="31" t="s">
-        <v>431</v>
+      <c r="I31" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="32" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -6341,8 +6359,8 @@
       <c r="H32" s="15">
         <v>3</v>
       </c>
-      <c r="I32" s="31" t="s">
-        <v>431</v>
+      <c r="I32" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -6370,12 +6388,12 @@
       <c r="H33" s="17">
         <v>4</v>
       </c>
-      <c r="I33" s="31" t="s">
-        <v>431</v>
+      <c r="I33" s="67" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A34" s="54" t="s">
+      <c r="A34" s="52" t="s">
         <v>355</v>
       </c>
       <c r="B34" s="53"/>
@@ -6390,7 +6408,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="52" t="s">
+      <c r="A36" s="54" t="s">
         <v>357</v>
       </c>
       <c r="B36" s="53"/>
@@ -6808,7 +6826,7 @@
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="54" t="s">
+      <c r="A51" s="52" t="s">
         <v>355</v>
       </c>
       <c r="B51" s="53"/>
@@ -6823,7 +6841,7 @@
       </c>
     </row>
     <row r="53" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="52" t="s">
+      <c r="A53" s="54" t="s">
         <v>358</v>
       </c>
       <c r="B53" s="53"/>
@@ -7560,7 +7578,7 @@
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A79" s="54" t="s">
+      <c r="A79" s="52" t="s">
         <v>355</v>
       </c>
       <c r="B79" s="53"/>
@@ -7575,7 +7593,7 @@
       </c>
     </row>
     <row r="81" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="52" t="s">
+      <c r="A81" s="54" t="s">
         <v>359</v>
       </c>
       <c r="B81" s="53"/>
@@ -7964,7 +7982,7 @@
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A95" s="54" t="s">
+      <c r="A95" s="52" t="s">
         <v>355</v>
       </c>
       <c r="B95" s="53"/>
@@ -7979,7 +7997,7 @@
       </c>
     </row>
     <row r="97" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="52" t="s">
+      <c r="A97" s="54" t="s">
         <v>360</v>
       </c>
       <c r="B97" s="53"/>
@@ -8078,7 +8096,7 @@
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A101" s="54" t="s">
+      <c r="A101" s="52" t="s">
         <v>355</v>
       </c>
       <c r="B101" s="53"/>
@@ -8109,6 +8127,7 @@
   </mergeCells>
   <phoneticPr fontId="10" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8129,7 +8148,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="58" t="s">
         <v>361</v>
       </c>
       <c r="B1" s="56"/>
@@ -8374,7 +8393,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="58" t="s">
+      <c r="A10" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B10" s="56"/>
@@ -8401,7 +8420,7 @@
       <c r="I11" s="38"/>
     </row>
     <row r="12" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="55" t="s">
+      <c r="A12" s="58" t="s">
         <v>363</v>
       </c>
       <c r="B12" s="56"/>
@@ -8699,7 +8718,7 @@
       <c r="H22" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="I22" s="41" t="s">
+      <c r="I22" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -8728,7 +8747,7 @@
       <c r="H23" s="34" t="s">
         <v>139</v>
       </c>
-      <c r="I23" s="41" t="s">
+      <c r="I23" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -8791,7 +8810,7 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A26" s="58" t="s">
+      <c r="A26" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B26" s="56"/>
@@ -8818,7 +8837,7 @@
       <c r="I27" s="38"/>
     </row>
     <row r="28" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="55" t="s">
+      <c r="A28" s="58" t="s">
         <v>364</v>
       </c>
       <c r="B28" s="56"/>
@@ -9058,7 +9077,7 @@
       <c r="H36" s="34" t="s">
         <v>51</v>
       </c>
-      <c r="I36" s="41" t="s">
+      <c r="I36" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -9150,7 +9169,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A40" s="58" t="s">
+      <c r="A40" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B40" s="56"/>
@@ -9177,7 +9196,7 @@
       <c r="I41" s="38"/>
     </row>
     <row r="42" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="55" t="s">
+      <c r="A42" s="58" t="s">
         <v>365</v>
       </c>
       <c r="B42" s="56"/>
@@ -9330,7 +9349,7 @@
       <c r="H47" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="I47" s="41" t="s">
+      <c r="I47" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -9359,7 +9378,7 @@
       <c r="H48" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="I48" s="41" t="s">
+      <c r="I48" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -9654,7 +9673,7 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="58" t="s">
+      <c r="A59" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B59" s="56"/>
@@ -9681,7 +9700,7 @@
       <c r="I60" s="38"/>
     </row>
     <row r="61" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="55" t="s">
+      <c r="A61" s="58" t="s">
         <v>366</v>
       </c>
       <c r="B61" s="56"/>
@@ -9776,7 +9795,7 @@
       <c r="H64" s="39" t="s">
         <v>30</v>
       </c>
-      <c r="I64" s="41" t="s">
+      <c r="I64" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -9805,7 +9824,7 @@
       <c r="H65" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="I65" s="41" t="s">
+      <c r="I65" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -9834,7 +9853,7 @@
       <c r="H66" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="I66" s="41" t="s">
+      <c r="I66" s="68" t="s">
         <v>431</v>
       </c>
     </row>
@@ -10535,7 +10554,7 @@
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A91" s="58" t="s">
+      <c r="A91" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B91" s="56"/>
@@ -10562,7 +10581,7 @@
       <c r="I92" s="38"/>
     </row>
     <row r="93" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="55" t="s">
+      <c r="A93" s="58" t="s">
         <v>367</v>
       </c>
       <c r="B93" s="56"/>
@@ -10633,7 +10652,7 @@
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A96" s="58" t="s">
+      <c r="A96" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B96" s="56"/>
@@ -10660,7 +10679,7 @@
       <c r="I97" s="46"/>
     </row>
     <row r="98" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="55" t="s">
+      <c r="A98" s="58" t="s">
         <v>368</v>
       </c>
       <c r="B98" s="56"/>
@@ -10731,7 +10750,7 @@
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A101" s="58" t="s">
+      <c r="A101" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B101" s="56"/>
@@ -10758,7 +10777,7 @@
       <c r="I102" s="38"/>
     </row>
     <row r="103" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A103" s="55" t="s">
+      <c r="A103" s="58" t="s">
         <v>369</v>
       </c>
       <c r="B103" s="56"/>
@@ -10916,7 +10935,7 @@
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A109" s="58" t="s">
+      <c r="A109" s="55" t="s">
         <v>362</v>
       </c>
       <c r="B109" s="56"/>
@@ -11054,7 +11073,7 @@
       </c>
     </row>
     <row r="4" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>386</v>
       </c>
       <c r="B4" s="53"/>
@@ -11607,7 +11626,7 @@
       </c>
     </row>
     <row r="24" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="52" t="s">
+      <c r="A24" s="54" t="s">
         <v>392</v>
       </c>
       <c r="B24" s="53"/>
@@ -11645,7 +11664,7 @@
       <c r="J25" s="22"/>
       <c r="K25" s="22"/>
       <c r="L25" s="22"/>
-      <c r="M25" s="31" t="s">
+      <c r="M25" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11672,7 +11691,7 @@
       <c r="J26" s="22"/>
       <c r="K26" s="22"/>
       <c r="L26" s="22"/>
-      <c r="M26" s="31" t="s">
+      <c r="M26" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11699,7 +11718,7 @@
       <c r="J27" s="22"/>
       <c r="K27" s="22"/>
       <c r="L27" s="22"/>
-      <c r="M27" s="31" t="s">
+      <c r="M27" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11726,7 +11745,7 @@
       <c r="J28" s="22"/>
       <c r="K28" s="22"/>
       <c r="L28" s="22"/>
-      <c r="M28" s="31" t="s">
+      <c r="M28" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11753,7 +11772,7 @@
       <c r="J29" s="22"/>
       <c r="K29" s="22"/>
       <c r="L29" s="22"/>
-      <c r="M29" s="31" t="s">
+      <c r="M29" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11780,7 +11799,7 @@
       <c r="J30" s="22"/>
       <c r="K30" s="22"/>
       <c r="L30" s="22"/>
-      <c r="M30" s="31" t="s">
+      <c r="M30" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11807,7 +11826,7 @@
       <c r="J31" s="47"/>
       <c r="K31" s="22"/>
       <c r="L31" s="22"/>
-      <c r="M31" s="31" t="s">
+      <c r="M31" s="67" t="s">
         <v>431</v>
       </c>
     </row>
@@ -11834,12 +11853,12 @@
       <c r="J32" s="47"/>
       <c r="K32" s="22"/>
       <c r="L32" s="22"/>
-      <c r="M32" s="31" t="s">
+      <c r="M32" s="67" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="52" t="s">
+      <c r="A33" s="54" t="s">
         <v>393</v>
       </c>
       <c r="B33" s="53"/>
@@ -12206,7 +12225,7 @@
       </c>
     </row>
     <row r="47" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="52" t="s">
+      <c r="A47" s="54" t="s">
         <v>394</v>
       </c>
       <c r="B47" s="53"/>
@@ -12870,7 +12889,7 @@
       </c>
     </row>
     <row r="72" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="52" t="s">
+      <c r="A72" s="54" t="s">
         <v>395</v>
       </c>
       <c r="B72" s="53"/>
@@ -13210,7 +13229,7 @@
       </c>
     </row>
     <row r="85" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="52" t="s">
+      <c r="A85" s="54" t="s">
         <v>396</v>
       </c>
       <c r="B85" s="53"/>

</xml_diff>

<commit_message>
docs(schedule): 更新工作分配表 — T-041/T-042 完成、T-090 部分完成
依 CHANGELOG 與 git log 校正 rank-service 與壓測進度：
- T-041 好友排行榜、T-042 排行榜查詢 API → ✅ 已完成
- T-090 JMeter 壓測腳本 → ⚠️ 部分完成（腳本已交付，實測阻塞於 T-032）

三個工作表（工作總覽／依職責分工／Sprint 時程甘特）同步更新狀態與配色。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -2688,9 +2688,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="J36" s="34" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="J36" s="32" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -2740,9 +2740,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="J37" s="34" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="J37" s="32" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -4196,9 +4196,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="J65" s="34" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="J65" s="33" t="inlineStr">
+        <is>
+          <t>⚠️ 部分完成</t>
         </is>
       </c>
     </row>
@@ -6782,6 +6782,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
     <row r="24" ht="19.5" customHeight="1" s="54">
       <c r="A24" s="68" t="inlineStr">
         <is>
@@ -7207,6 +7208,7 @@
         <v/>
       </c>
     </row>
+    <row r="35"/>
     <row r="36" ht="19.5" customHeight="1" s="54">
       <c r="A36" s="68" t="inlineStr">
         <is>
@@ -7857,6 +7859,7 @@
         <v/>
       </c>
     </row>
+    <row r="52"/>
     <row r="53" ht="19.5" customHeight="1" s="54">
       <c r="A53" s="68" t="inlineStr">
         <is>
@@ -8085,9 +8088,9 @@
       <c r="H58" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="I58" s="34" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="I58" s="32" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8130,9 +8133,9 @@
       <c r="H59" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="I59" s="34" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="I59" s="32" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8760,9 +8763,9 @@
       <c r="H73" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="I73" s="34" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="I73" s="33" t="inlineStr">
+        <is>
+          <t>⚠️ 部分完成</t>
         </is>
       </c>
     </row>
@@ -9002,6 +9005,7 @@
         <v/>
       </c>
     </row>
+    <row r="80"/>
     <row r="81" ht="19.5" customHeight="1" s="54">
       <c r="A81" s="68" t="inlineStr">
         <is>
@@ -9607,6 +9611,7 @@
         <v/>
       </c>
     </row>
+    <row r="96"/>
     <row r="97" ht="19.5" customHeight="1" s="54">
       <c r="A97" s="68" t="inlineStr">
         <is>
@@ -11775,9 +11780,9 @@
           <t>4</t>
         </is>
       </c>
-      <c r="I49" s="46" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="I49" s="40" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -11822,9 +11827,9 @@
           <t>3</t>
         </is>
       </c>
-      <c r="I50" s="46" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="I50" s="40" t="inlineStr">
+        <is>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -13727,9 +13732,9 @@
           <t>5</t>
         </is>
       </c>
-      <c r="I95" s="46" t="inlineStr">
-        <is>
-          <t>⬜ 未開始</t>
+      <c r="I95" s="41" t="inlineStr">
+        <is>
+          <t>⚠️ 部分完成</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(stage): 更新工作分配表進度 — T-002/050/051/052/053/105/106 標記完成
依本分支已完成並驗證的任務，將工作總覽/依職責分工/Sprint甘特/視覺化甘特四個分頁的狀態更新為「✅ 已完成」（T-041/T-042 補齊視覺化甘特分頁）。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -1030,7 +1030,7 @@
       </c>
       <c r="J4" s="30" t="inlineStr">
         <is>
-          <t>⚠️ 部分完成</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
       </c>
       <c r="J41" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -3006,7 +3006,7 @@
       </c>
       <c r="J42" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -3058,7 +3058,7 @@
       </c>
       <c r="J43" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -3110,7 +3110,7 @@
       </c>
       <c r="J44" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -4815,7 +4815,7 @@
       </c>
       <c r="J78" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -4865,7 +4865,7 @@
       </c>
       <c r="J79" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="I55" s="30" t="inlineStr">
         <is>
-          <t>⚠️ 部分完成</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8319,7 +8319,7 @@
       </c>
       <c r="I63" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8364,7 +8364,7 @@
       </c>
       <c r="I64" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8409,7 +8409,7 @@
       </c>
       <c r="I65" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8454,7 +8454,7 @@
       </c>
       <c r="I66" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="I77" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -8994,7 +8994,7 @@
       </c>
       <c r="I78" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -10010,7 +10010,7 @@
       </c>
       <c r="I5" s="37" t="inlineStr">
         <is>
-          <t>⚠️ 部分完成</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -12669,7 +12669,7 @@
       </c>
       <c r="I70" s="41" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -12716,7 +12716,7 @@
       </c>
       <c r="I71" s="41" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -12763,7 +12763,7 @@
       </c>
       <c r="I72" s="41" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -12810,7 +12810,7 @@
       </c>
       <c r="I73" s="41" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -13511,7 +13511,7 @@
       </c>
       <c r="I88" s="41" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -13556,7 +13556,7 @@
       </c>
       <c r="I89" s="41" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -15923,7 +15923,7 @@
       <c r="L48" s="22" t="n"/>
       <c r="M48" s="30" t="inlineStr">
         <is>
-          <t>⚠️ 部分完成</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16034,7 +16034,7 @@
       <c r="L51" s="22" t="n"/>
       <c r="M51" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
       <c r="L52" s="22" t="n"/>
       <c r="M52" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16182,7 +16182,7 @@
       <c r="L55" s="22" t="n"/>
       <c r="M55" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16219,7 +16219,7 @@
       <c r="L56" s="22" t="n"/>
       <c r="M56" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16330,7 +16330,7 @@
       <c r="L59" s="22" t="n"/>
       <c r="M59" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16367,7 +16367,7 @@
       <c r="L60" s="22" t="n"/>
       <c r="M60" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16441,7 +16441,7 @@
       <c r="L62" s="22" t="n"/>
       <c r="M62" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -16478,7 +16478,7 @@
       <c r="L63" s="22" t="n"/>
       <c r="M63" s="31" t="inlineStr">
         <is>
-          <t>⬜ 未開始</t>
+          <t>✅ 已完成</t>
         </is>
       </c>
     </row>
@@ -17373,6 +17373,7 @@
       <c r="K89" s="64" t="n"/>
       <c r="L89" s="65" t="n"/>
     </row>
+    <row r="90"/>
     <row r="91" ht="22.8" customHeight="1" s="55">
       <c r="A91" s="25" t="inlineStr">
         <is>
@@ -17484,6 +17485,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="14.4" customHeight="1" s="55">
       <c r="A6" s="68" t="inlineStr">
         <is>
@@ -17551,6 +17553,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13" ht="14.4" customHeight="1" s="55">
       <c r="A13" s="68" t="inlineStr">
         <is>
@@ -17594,6 +17597,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="14.4" customHeight="1" s="55">
       <c r="A18" s="51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(admin-service): 完成 T-054 異常玩家偵測
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -3637,7 +3637,7 @@
         <v>30</v>
       </c>
       <c r="J46" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -7671,7 +7671,7 @@
         <v>5</v>
       </c>
       <c r="I68" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -10539,7 +10539,7 @@
         <v>30</v>
       </c>
       <c r="I75" s="41" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -13284,7 +13284,7 @@
       <c r="K69" s="46"/>
       <c r="L69" s="22"/>
       <c r="M69" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fix(admin-service): 完成 T-055 GM 手動發幣
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -3669,7 +3669,7 @@
         <v>18</v>
       </c>
       <c r="J47" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -7700,7 +7700,7 @@
         <v>3</v>
       </c>
       <c r="I69" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -10568,7 +10568,7 @@
         <v>18</v>
       </c>
       <c r="I76" s="41" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -13311,7 +13311,7 @@
       <c r="K70" s="46"/>
       <c r="L70" s="22"/>
       <c r="M70" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
docs(notification): 更新 T-073 工作分配表狀態
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -3925,7 +3925,7 @@
         <v>18</v>
       </c>
       <c r="J55" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -7816,7 +7816,7 @@
         <v>3</v>
       </c>
       <c r="I73" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -10684,7 +10684,7 @@
         <v>18</v>
       </c>
       <c r="I80" s="41" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="81" spans="1:9" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -13203,7 +13203,7 @@
       <c r="K66" s="22"/>
       <c r="L66" s="22"/>
       <c r="M66" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
docs(devops): 更新 T-091 工作分配表狀態
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -4418,7 +4418,7 @@
         <v>18</v>
       </c>
       <c r="J67" s="30" t="s">
-        <v>272</v>
+        <v>19</v>
       </c>
     </row>
     <row r="68" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -7983,7 +7983,7 @@
         <v>3</v>
       </c>
       <c r="I75" s="30" t="s">
-        <v>272</v>
+        <v>19</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -11308,7 +11308,7 @@
         <v>18</v>
       </c>
       <c r="I101" s="37" t="s">
-        <v>272</v>
+        <v>19</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.3">
@@ -13447,7 +13447,7 @@
       </c>
       <c r="L71" s="22"/>
       <c r="M71" s="30" t="s">
-        <v>272</v>
+        <v>19</v>
       </c>
     </row>
     <row r="72" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat(devops): 完成 T-092 Swagger 文件聚合
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -4450,7 +4450,7 @@
         <v>18</v>
       </c>
       <c r="J68" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -8012,7 +8012,7 @@
         <v>3</v>
       </c>
       <c r="I76" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -10996,7 +10996,7 @@
         <v>18</v>
       </c>
       <c r="I87" s="41" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="88" spans="1:9" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -13474,7 +13474,7 @@
       <c r="K72" s="46"/>
       <c r="L72" s="22"/>
       <c r="M72" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
feat(devops): complete T-092 Swagger OpenAPI aggregation
Merge PR #116 into develop
</commit_message>
<xml_diff>
--- a/docs/幸運星幣城_工作分配表.xlsx
+++ b/docs/幸運星幣城_工作分配表.xlsx
@@ -4450,7 +4450,7 @@
         <v>18</v>
       </c>
       <c r="J68" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="69" spans="1:10" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -8012,7 +8012,7 @@
         <v>3</v>
       </c>
       <c r="I76" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -10996,7 +10996,7 @@
         <v>18</v>
       </c>
       <c r="I87" s="41" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="88" spans="1:9" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
@@ -13474,7 +13474,7 @@
       <c r="K72" s="46"/>
       <c r="L72" s="22"/>
       <c r="M72" s="31" t="s">
-        <v>191</v>
+        <v>19</v>
       </c>
     </row>
     <row r="73" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>